<commit_message>
Revise initial system test checklist for current leave rules.
Co-authored-by: kdtdev06 <kdtdev06@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/Leave_Forms_Initial_System_Test_Checklist.xlsx
+++ b/docs/Leave_Forms_Initial_System_Test_Checklist.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'How to Use'!$1:$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Checklist'!$A$4:$J$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Checklist'!$A$4:$J$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Test Checklist'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -853,9 +853,9 @@
     <row r="24" ht="86" customHeight="1">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Most real updates are sent by email, not by the bell icon.
+          <t>Real updates are sent by email.
 If email is not turned on in this environment, write that in Remarks and mark the email part Blocked — do not fail the whole leave if the screen still worked.
-The bell icon is still under development. Sample messages there are not a fail.</t>
+The bell icon in the header is not a finished feature. It should be removed from the final screens. Do not test it as a working notification list.</t>
         </is>
       </c>
       <c r="C24" s="6" t="n"/>
@@ -868,12 +868,16 @@
       </c>
       <c r="C26" s="4" t="n"/>
     </row>
-    <row r="27" ht="128" customHeight="1">
+    <row r="27" ht="130" customHeight="1">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>• For Vacation Leave, use 1 or 2 working days. Three or more days in a row must start at least one month later, or the form will stop you.
+          <t>• When you file Vacation Leave for yourself, use 1 or 2 working days first. Three or more consecutive working days must start at least one month later, or the form will stop you.
+• An approver filing leave for a team member can file 3 or more Vacation Leave days even if the start date is less than one month away. That is expected.
+• Long Leave is available. It must last between 1 and 3 calendar months, needs a supporting document, and is always unpaid. There is no 5-year service rule and no waiting period after a previous Long Leave.
+• You cannot file a second Long Leave while another Long Leave is still waiting for approval.
 • Do not pick dates that overlap another open or approved leave.
-• Avoid weekends and holidays for Vacation, Sick, Emergency, and Paternity Leave.
+• Avoid weekends and holidays for Vacation, Sick, Emergency, and Paternity Leave. Long Leave, PTB, and Maternity count every calendar day.
+• Paternity Leave needs a Paternity Notification Form attached.
 • Keep a simple screenshot naming style, for example: 2.1-after-submit.png, 2.4-approver-email.png.
 • After the run, fill in the Test Run Summary sheet.</t>
         </is>
@@ -942,7 +946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -976,7 +980,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Perform the items from top to bottom. Start on Dashboard after access is already given. Do not test Sign in. For unfinished items, choose Pending Development — that is not a Fail. Write what you saw in Actual Result. Attach screenshot names under Test Evidence.</t>
+          <t>Revised to match the current system. Perform the items from top to bottom. Start on Dashboard after access is already given. Do not test Sign in. For unfinished items, choose Pending Development — that is not a Fail. Write what you saw in Actual Result. Attach screenshot names under Test Evidence.</t>
         </is>
       </c>
       <c r="B2" s="6" t="n"/>
@@ -1376,79 +1380,124 @@
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
     </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="15" t="n"/>
-      <c r="B13" s="16" t="inlineStr">
+    <row r="13" ht="74" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>File your own Vacation Leave of 3 or more days too soon</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>Go to File Leave.
+Leave Type: Vacation Leave. Day Type: Whole day.
+Pick 3 or more consecutive working days that start less than one month from today.
+Enter a Reason and click Submit Request.</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>The form does not allow you to submit.
+A warning explains that leave of 3 or more consecutive days must be filed at least 1 month before the start date.
+No new leave request is created.</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>None — the request should not be sent.</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr"/>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  3.  Reject a Vacation Leave    —    Use a different set of dates so this does not overlap the approved leave.</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="15" t="n"/>
-      <c r="J13" s="15" t="n"/>
-    </row>
-    <row r="14" ht="56" customHeight="1">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
+      <c r="G14" s="15" t="n"/>
+      <c r="H14" s="15" t="n"/>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="n"/>
+    </row>
+    <row r="15" ht="56" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>File a second Vacation Leave (for reject)</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>File another short Vacation Leave (1–2 working days) on new dates, same way as 2.1.</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>The request is submitted and shows Pending Approval. Reserved credits increase again.</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F15" s="18" t="inlineStr">
         <is>
           <t>The approver should receive another waiting-for-approval email.</t>
         </is>
       </c>
-      <c r="G14" s="11" t="inlineStr"/>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr"/>
-      <c r="J14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="G15" s="11" t="inlineStr"/>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Approver rejects the leave</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>Approver</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Open Leave Approvals → Pending Approvals.
 Click Review on the new request.
@@ -1457,50 +1506,50 @@
 Confirm.</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>A success message appears: Leave request rejected successfully.
 On All Leave Requests the status is Rejected.
 The request is gone from Pending Approvals.</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>The employee should receive an email that the leave request has been rejected.</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr"/>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr"/>
-      <c r="J15" s="11" t="inlineStr"/>
-    </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="G16" s="11" t="inlineStr"/>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
+      <c r="J16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Employee confirms the rejected leave</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>Open the rejected request from the Dashboard.
 Check Vacation Leave balances and Activity Log.</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Status is Rejected.
 The reserved days are given back (available days return).
@@ -1508,98 +1557,99 @@
 Activity Log shows the rejection.</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>The rejection email from step 3.2 should have arrived.</t>
         </is>
       </c>
-      <c r="G16" s="11" t="inlineStr"/>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
-      <c r="J16" s="11" t="inlineStr"/>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="15" t="n"/>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="G17" s="11" t="inlineStr"/>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr"/>
+      <c r="J17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  4.  Edit or cancel a leave that is still waiting    —    These only work while the leave is still Pending Approval and nobody has approved or rejected it yet. File a new short Vacation Leave first if you do not have one waiting.</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="15" t="n"/>
-      <c r="H17" s="15" t="n"/>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-    </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="n"/>
+      <c r="G18" s="15" t="n"/>
+      <c r="H18" s="15" t="n"/>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="88" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Edit a pending leave</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>Open a leave that is still Pending Approval.
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>Open a leave that you filed yourself and that is still Pending Approval.
 Click Edit Request.
 Change the dates and/or the reason.
 Click Save Changes, then confirm Save.</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E19" s="18" t="inlineStr">
         <is>
           <t>A success message appears: Leave request updated successfully.
 The details page shows the new dates and reason.
-Status is still Pending Approval.</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
+Status is still Pending Approval.
+If the leave was filed for you by someone else, Edit Request is not available — see 8.3.</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
         <is>
           <t>The waiting approver should receive an email that the leave request was updated and still needs approval.</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr"/>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
-      <c r="J18" s="11" t="inlineStr"/>
-    </row>
-    <row r="19" ht="74" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="G19" s="11" t="inlineStr"/>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I19" s="11" t="inlineStr"/>
+      <c r="J19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20" ht="74" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Cancel a pending leave</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D20" s="21" t="inlineStr">
         <is>
           <t>Open a leave that is still Pending Approval (use a request you do not need to keep).
 Click Cancel Request.
@@ -1607,60 +1657,60 @@
 Click Cancel Request on the confirmation.</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>A success message appears: Leave request cancelled successfully.
 Status becomes Cancelled.
 Reserved days are given back to available credits.</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="F20" s="21" t="inlineStr">
         <is>
           <t>The designated approver should receive an email that the leave request was cancelled.</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr"/>
-      <c r="H19" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I19" s="11" t="inlineStr"/>
-      <c r="J19" s="11" t="inlineStr"/>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="15" t="n"/>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr"/>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
+      <c r="J20" s="11" t="inlineStr"/>
+    </row>
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  5.  File a Sick Leave — Admin reviews it    —    Sick Leave is reviewed by Admin, not by the team approver. Team leaders may be copied on the email but should not be able to approve it.</t>
         </is>
       </c>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="15" t="n"/>
-      <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
-    </row>
-    <row r="21" ht="74" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="n"/>
+      <c r="G21" s="15" t="n"/>
+      <c r="H21" s="15" t="n"/>
+      <c r="I21" s="15" t="n"/>
+      <c r="J21" s="15" t="n"/>
+    </row>
+    <row r="22" ht="74" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>File Sick Leave</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D21" s="18" t="inlineStr">
+      <c r="D22" s="18" t="inlineStr">
         <is>
           <t>Go to File Leave.
 Leave Type: Sick Leave.
@@ -1670,45 +1720,45 @@
 Click Submit Request, then Submit.</t>
         </is>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E22" s="18" t="inlineStr">
         <is>
           <t>The request is submitted successfully.
 It appears on the Dashboard as Pending Approval.
 If you had Sick Leave credits, some may now show as reserved.</t>
         </is>
       </c>
-      <c r="F21" s="18" t="inlineStr">
+      <c r="F22" s="18" t="inlineStr">
         <is>
           <t>Admin should receive an email that a Sick Leave is waiting for approval, with the medical certificate attached.
 The team approver may be copied on that email, but they should not approve this request.</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr"/>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I21" s="11" t="inlineStr"/>
-      <c r="J21" s="11" t="inlineStr"/>
-    </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="G22" s="11" t="inlineStr"/>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
+      <c r="J22" s="11" t="inlineStr"/>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>Admin opens the Sick Leave for review</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D23" s="21" t="inlineStr">
         <is>
           <t>Switch to the Admin user.
 Open Leave Requests.
@@ -1716,143 +1766,143 @@
 Find the Sick Leave and click Review.</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>The Sick Leave is in the Pending Validation list.
 The review page shows the details and the attached medical certificate.
 Approve and Reject buttons are available.</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F23" s="21" t="inlineStr">
         <is>
           <t>This should match the Admin email from step 5.1.</t>
         </is>
       </c>
-      <c r="G22" s="11" t="inlineStr"/>
-      <c r="H22" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
-      <c r="J22" s="11" t="inlineStr"/>
-    </row>
-    <row r="23" ht="56" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr"/>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I23" s="11" t="inlineStr"/>
+      <c r="J23" s="11" t="inlineStr"/>
+    </row>
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Admin approves the Sick Leave</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>Click Approve and confirm.</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E24" s="18" t="inlineStr">
         <is>
           <t>A success message appears: Leave request approved successfully.
 On All Leave Requests the status is Approved.</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>The employee should receive an email that the leave request has been approved.</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr"/>
-      <c r="H23" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I23" s="11" t="inlineStr"/>
-      <c r="J23" s="11" t="inlineStr"/>
-    </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr"/>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
+      <c r="J24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Employee confirms the approved Sick Leave</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Open the Sick Leave from the Dashboard.</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>Status is Approved.
 Request Conversion is not shown (only Vacation Leave can be converted).
 The medical certificate can still be viewed.</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>The approval email from step 5.3 should have arrived.</t>
         </is>
       </c>
-      <c r="G24" s="11" t="inlineStr"/>
-      <c r="H24" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr"/>
-      <c r="J24" s="11" t="inlineStr"/>
-    </row>
-    <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="15" t="n"/>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr"/>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I25" s="11" t="inlineStr"/>
+      <c r="J25" s="11" t="inlineStr"/>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="15" t="n"/>
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  6.  Other leave types    —    Use the same File Leave page. Admin reviews these the same way as Sick Leave (Pending Validation → Review → Approve or Reject). Skip a type if it does not apply to the test employee.</t>
         </is>
       </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="15" t="n"/>
-      <c r="H25" s="15" t="n"/>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-    </row>
-    <row r="26" ht="88" customHeight="1">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="n"/>
+      <c r="G26" s="15" t="n"/>
+      <c r="H26" s="15" t="n"/>
+      <c r="I26" s="15" t="n"/>
+      <c r="J26" s="15" t="n"/>
+    </row>
+    <row r="27" ht="88" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>File Emergency Leave</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Employee, then Admin</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>File Leave → Emergency Leave.
 Day Type is Whole day only.
@@ -1861,44 +1911,44 @@
 Submit, then as Admin approve it from Pending Validation.</t>
         </is>
       </c>
-      <c r="E26" s="18" t="inlineStr">
+      <c r="E27" s="18" t="inlineStr">
         <is>
           <t>The request is submitted if you have enough Emergency Leave credits.
 If you do not have enough credits, the form blocks you (this type cannot go unpaid).
 After Admin approves, status is Approved.</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>Admin receives an email (supporting document attached). Team approver may be copied. After approval, the employee receives an approval email.</t>
         </is>
       </c>
-      <c r="G26" s="11" t="inlineStr"/>
-      <c r="H26" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr"/>
-      <c r="J26" s="11" t="inlineStr"/>
-    </row>
-    <row r="27" ht="96" customHeight="1">
-      <c r="A27" s="20" t="inlineStr">
+      <c r="G27" s="11" t="inlineStr"/>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr"/>
+      <c r="J27" s="11" t="inlineStr"/>
+    </row>
+    <row r="28" ht="96" customHeight="1">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>File PTB Leave</t>
         </is>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>Employee, then Admin</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D28" s="21" t="inlineStr">
         <is>
           <t>File Leave → PTB Leave.
 Day Type is Whole day only.
@@ -1908,42 +1958,42 @@
 Submit, then Admin approves from Pending Validation.</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E28" s="21" t="inlineStr">
         <is>
           <t>Submitted if credits are enough. After Admin approval, status is Approved.</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="F28" s="21" t="inlineStr">
         <is>
           <t>Same pattern as Sick Leave: email to Admin with the file; approval email to the employee.</t>
         </is>
       </c>
-      <c r="G27" s="11" t="inlineStr"/>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I27" s="11" t="inlineStr"/>
-      <c r="J27" s="11" t="inlineStr"/>
-    </row>
-    <row r="28" ht="88" customHeight="1">
-      <c r="A28" s="17" t="inlineStr">
+      <c r="G28" s="11" t="inlineStr"/>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
+      <c r="J28" s="11" t="inlineStr"/>
+    </row>
+    <row r="29" ht="88" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>File Maternity Leave</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Employee (female), then Admin</t>
         </is>
       </c>
-      <c r="D28" s="18" t="inlineStr">
+      <c r="D29" s="18" t="inlineStr">
         <is>
           <t>As a female employee, File Leave → Maternity Leave.
 Pick a Start Date. The End Date should fill in automatically (105 calendar days).
@@ -1951,145 +2001,159 @@
 Submit, then Admin approves from Pending Validation.</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="E29" s="18" t="inlineStr">
         <is>
           <t>Maternity Leave appears in the leave type list only for a female employee.
 After submit, status is Pending Approval.
 After Admin approves, status is Approved.</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>Admin receives an email (no file). After approval, the employee receives an approval email.</t>
         </is>
       </c>
-      <c r="G28" s="11" t="inlineStr"/>
-      <c r="H28" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
-      <c r="J28" s="11" t="inlineStr"/>
-    </row>
-    <row r="29" ht="88" customHeight="1">
-      <c r="A29" s="20" t="inlineStr">
+      <c r="G29" s="11" t="inlineStr"/>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr"/>
+      <c r="J29" s="11" t="inlineStr"/>
+    </row>
+    <row r="30" ht="96" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B29" s="21" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>File Paternity Leave</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C30" s="21" t="inlineStr">
         <is>
           <t>Employee (male), then Admin</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t>As a male employee, File Leave → Paternity Leave.
 Pick a Start Date that is a working day. The End Date should fill in automatically (7 working days).
-No attachment is required.
+Attach a Paternity Notification Form (PDF, JPG, or PNG).
 Submit, then Admin approves from Pending Validation.</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E30" s="21" t="inlineStr">
         <is>
           <t>Paternity Leave appears in the leave type list only for a male employee.
+A Paternity Notification Form is required.
 After submit, status is Pending Approval.
 After Admin approves, status is Approved.</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
-        <is>
-          <t>Admin receives an email (no file). After approval, the employee receives an approval email.</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="inlineStr"/>
-      <c r="H29" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I29" s="11" t="inlineStr"/>
-      <c r="J29" s="11" t="inlineStr"/>
-    </row>
-    <row r="30" ht="56" customHeight="1">
-      <c r="A30" s="22" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="B30" s="23" t="inlineStr">
-        <is>
-          <t>File Long Leave</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>Employee</t>
-        </is>
-      </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>Open File Leave and look at the Leave Type list for Long Leave.</t>
-        </is>
-      </c>
-      <c r="E30" s="23" t="inlineStr">
-        <is>
-          <t>Long Leave is not in the File Leave list yet. You cannot file it from the screen.</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>Admin receives an email with the form attached. The team approver may be copied. After approval, the employee receives an approval email.</t>
         </is>
       </c>
       <c r="G30" s="11" t="inlineStr"/>
-      <c r="H30" s="24" t="inlineStr">
-        <is>
-          <t>Pending Development</t>
+      <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="11" t="inlineStr"/>
     </row>
-    <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="15" t="n"/>
-      <c r="B31" s="16" t="inlineStr">
+    <row r="31" ht="96" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>File Long Leave</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Employee, then Admin</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>Go to File Leave.
+Leave Type: Long Leave.
+Day Type is Whole day only.
+Pick a Start Date. The End Date must be at least 1 calendar month and at most 3 calendar months later (for example, start 15 September → end from 14 October through 14 December).
+Enter a Reason.
+Attach a supporting document (PDF, JPG, or PNG).
+Submit Request, then as Admin open Leave Requests → Pending Validation, click Review, and Approve.
+If you already have a Long Leave still waiting for approval, try filing another one.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Long Leave is in the Leave Type list.
+There is no 5-year service requirement. An employee with less than 5 years of service can file it.
+A previous approved Long Leave does not block a new one.
+The leave is unpaid. Vacation or Sick Leave credits do not go down.
+You cannot file a second Long Leave while another is still Pending Approval.
+After submit, status is Pending Approval. After Admin approves, status is Approved.
+On the team calendar, Long Leave can cover weekends and holidays.</t>
+        </is>
+      </c>
+      <c r="F31" s="18" t="inlineStr">
+        <is>
+          <t>Admin receives an email that a Long Leave is waiting for approval, with the supporting document attached. The team approver may be copied. After approval, the employee receives an approval email.</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr"/>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr"/>
+      <c r="J31" s="11" t="inlineStr"/>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="15" t="n"/>
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  7.  Convert an approved Vacation Leave to Sick Leave    —    Use the Vacation Leave that was approved in section 2. Only the person who took the leave can request this — not someone who filed it for them.</t>
         </is>
       </c>
-      <c r="C31" s="15" t="n"/>
-      <c r="D31" s="15" t="n"/>
-      <c r="E31" s="15" t="n"/>
-      <c r="F31" s="15" t="n"/>
-      <c r="G31" s="15" t="n"/>
-      <c r="H31" s="15" t="n"/>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-    </row>
-    <row r="32" ht="88" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="88" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>7.1</t>
         </is>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Request conversion to Sick Leave</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D32" s="18" t="inlineStr">
+      <c r="D33" s="18" t="inlineStr">
         <is>
           <t>Open the approved Vacation Leave.
 Click Request Conversion.
@@ -2099,230 +2163,230 @@
 Click Confirm, then Submit conversion.</t>
         </is>
       </c>
-      <c r="E32" s="18" t="inlineStr">
+      <c r="E33" s="18" t="inlineStr">
         <is>
           <t>A success message appears: Leave conversion submitted successfully.
 The leave status becomes Pending Conversion.</t>
         </is>
       </c>
-      <c r="F32" s="18" t="inlineStr">
+      <c r="F33" s="18" t="inlineStr">
         <is>
           <t>Admin should receive an email that a conversion is waiting for review, with the medical certificate attached. The team approver may be copied.</t>
         </is>
       </c>
-      <c r="G32" s="11" t="inlineStr"/>
-      <c r="H32" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
-      <c r="J32" s="11" t="inlineStr"/>
-    </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="20" t="inlineStr">
+      <c r="G33" s="11" t="inlineStr"/>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I33" s="11" t="inlineStr"/>
+      <c r="J33" s="11" t="inlineStr"/>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="B33" s="21" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Admin approves the conversion</t>
         </is>
       </c>
-      <c r="C33" s="21" t="inlineStr">
+      <c r="C34" s="21" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D34" s="21" t="inlineStr">
         <is>
           <t>Open Leave Requests → Pending Validation.
 Find the request shown as Vacation Leave to Sick Leave.
 Click Review, then Approve, and confirm.</t>
         </is>
       </c>
-      <c r="E33" s="21" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>A success message appears: Leave conversion request approved successfully.
 On All Leave Requests the status is Converted to SL.</t>
         </is>
       </c>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="F34" s="21" t="inlineStr">
         <is>
           <t>The employee should receive an email that the conversion was approved.</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr"/>
-      <c r="H33" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I33" s="11" t="inlineStr"/>
-      <c r="J33" s="11" t="inlineStr"/>
-    </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
+      <c r="G34" s="11" t="inlineStr"/>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr"/>
+      <c r="J34" s="11" t="inlineStr"/>
+    </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>Employee confirms the converted leave</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C35" s="18" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D35" s="18" t="inlineStr">
         <is>
           <t>Open the same leave from the Dashboard. Check leave balances.</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E35" s="18" t="inlineStr">
         <is>
           <t>Status is Converted to SL.
 Request Conversion is no longer shown.
 Vacation Leave days for that leave are given back, and Sick Leave days are deducted.</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F35" s="18" t="inlineStr">
         <is>
           <t>The conversion approval email from step 7.2 should have arrived.</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr"/>
-      <c r="H34" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I34" s="11" t="inlineStr"/>
-      <c r="J34" s="11" t="inlineStr"/>
-    </row>
-    <row r="35" ht="74" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr"/>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr"/>
+      <c r="J35" s="11" t="inlineStr"/>
+    </row>
+    <row r="36" ht="74" customHeight="1">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Admin rejects a conversion (optional)</t>
         </is>
       </c>
-      <c r="C35" s="21" t="inlineStr">
+      <c r="C36" s="21" t="inlineStr">
         <is>
           <t>Admin, then Employee</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D36" s="21" t="inlineStr">
         <is>
           <t>If you have another approved Vacation Leave, request conversion again.
 As Admin, open it from Pending Validation, click Reject, enter a reason, and confirm.
 As Employee, open the leave again.</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>After reject, the leave goes back to Approved (still Vacation Leave).
 Leave credits do not change because of the rejection.</t>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr">
+      <c r="F36" s="21" t="inlineStr">
         <is>
           <t>The employee should receive an email that the conversion was rejected.</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr"/>
-      <c r="H35" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I35" s="11" t="inlineStr"/>
-      <c r="J35" s="11" t="inlineStr"/>
-    </row>
-    <row r="36" ht="60" customHeight="1">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr"/>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I36" s="11" t="inlineStr"/>
+      <c r="J36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="22" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>Request conversion to Emergency Leave</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C37" s="23" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D36" s="23" t="inlineStr">
+      <c r="D37" s="23" t="inlineStr">
         <is>
           <t>On an approved Vacation Leave, click Request Conversion.
 Select Emergency Leave and click Continue.
 Fill in the reason and a document if asked, then try Confirm.</t>
         </is>
       </c>
-      <c r="E36" s="23" t="inlineStr">
+      <c r="E37" s="23" t="inlineStr">
         <is>
           <t>The page opens, but submission is not available yet.
 A message explains that Emergency Leave conversion is not available yet.</t>
         </is>
       </c>
-      <c r="F36" s="23" t="inlineStr">
+      <c r="F37" s="23" t="inlineStr">
         <is>
           <t>None — this is not connected yet.</t>
         </is>
       </c>
-      <c r="G36" s="11" t="inlineStr"/>
-      <c r="H36" s="24" t="inlineStr">
+      <c r="G37" s="11" t="inlineStr"/>
+      <c r="H37" s="24" t="inlineStr">
         <is>
           <t>Pending Development</t>
         </is>
       </c>
-      <c r="I36" s="11" t="inlineStr"/>
-      <c r="J36" s="11" t="inlineStr"/>
-    </row>
-    <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="15" t="n"/>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="I37" s="11" t="inlineStr"/>
+      <c r="J37" s="11" t="inlineStr"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="15" t="n"/>
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  8.  File leave for a team member    —    The approver files on behalf of someone in their group. A higher-level approver (or the usual approver for that person) still needs to approve it.</t>
         </is>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15" t="n"/>
-      <c r="G37" s="15" t="n"/>
-      <c r="H37" s="15" t="n"/>
-      <c r="I37" s="15" t="n"/>
-      <c r="J37" s="15" t="n"/>
-    </row>
-    <row r="38" ht="74" customHeight="1">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="C38" s="15" t="n"/>
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="15" t="n"/>
+      <c r="I38" s="15" t="n"/>
+      <c r="J38" s="15" t="n"/>
+    </row>
+    <row r="39" ht="74" customHeight="1">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>8.1</t>
         </is>
       </c>
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B39" s="18" t="inlineStr">
         <is>
           <t>File Vacation Leave for a member</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>Approver</t>
         </is>
       </c>
-      <c r="D38" s="18" t="inlineStr">
+      <c r="D39" s="18" t="inlineStr">
         <is>
           <t>Open File Leave for Member.
 Select the Group, then the Employee.
@@ -2330,60 +2394,150 @@
 Submit the request.</t>
         </is>
       </c>
-      <c r="E38" s="18" t="inlineStr">
+      <c r="E39" s="18" t="inlineStr">
         <is>
           <t>A success message appears.
 When you switch to that employee’s Dashboard, the leave is there as Pending Approval.
 The details show that it was filed by the approver, not by the employee.</t>
         </is>
       </c>
-      <c r="F38" s="18" t="inlineStr">
+      <c r="F39" s="18" t="inlineStr">
         <is>
           <t>The person who needs to approve that employee’s leave should receive the waiting-for-approval email.</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr"/>
-      <c r="H38" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I38" s="11" t="inlineStr"/>
-      <c r="J38" s="11" t="inlineStr"/>
-    </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="15" t="n"/>
-      <c r="B39" s="16" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr"/>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr"/>
+      <c r="J39" s="11" t="inlineStr"/>
+    </row>
+    <row r="40" ht="96" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t>File 3 or more Vacation Leave days for a member, less than one month in advance</t>
+        </is>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>Approver</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Open File Leave for Member.
+Select a Group and an Employee.
+Leave Type: Vacation Leave. Day Type: Whole day.
+Pick 3 or more consecutive working days that start less than one month from today.
+Enter a Reason and Submit Request.</t>
+        </is>
+      </c>
+      <c r="E40" s="21" t="inlineStr">
+        <is>
+          <t>The request is submitted successfully. The one-month advance rule does not apply when an approver files for a member.
+The leave appears on the member’s Dashboard as Pending Approval.
+Reserved Vacation Leave credits are held for the member, if they have enough credits. Extra days may be treated as unpaid.</t>
+        </is>
+      </c>
+      <c r="F40" s="21" t="inlineStr">
+        <is>
+          <t>The person who needs to approve that member’s leave should receive the waiting-for-approval email.</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr"/>
+      <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr"/>
+      <c r="J40" s="11" t="inlineStr"/>
+    </row>
+    <row r="41" ht="96" customHeight="1">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>Who can edit a leave filed for a member</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>Employee, then Approver who filed it</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>As the member, open the leave that was filed for you while it is still Pending Approval.
+Check whether Edit Request is available.
+Then switch to the approver who filed it and open the same leave if you can.</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>The member cannot edit a leave that someone else filed for them. Edit Request is not available (or is disabled).
+The member can still Cancel Request while it is Pending Approval.
+Only the person who filed it can edit it, and only while nobody has approved or rejected it yet.</t>
+        </is>
+      </c>
+      <c r="F41" s="18" t="inlineStr">
+        <is>
+          <t>If the filer edits it, the waiting approver should receive an updated-request email.</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr"/>
+      <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr"/>
+      <c r="J41" s="11" t="inlineStr"/>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="15" t="n"/>
+      <c r="B42" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  9.  Team Leave Calendar</t>
         </is>
       </c>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="15" t="n"/>
-      <c r="G39" s="15" t="n"/>
-      <c r="H39" s="15" t="n"/>
-      <c r="I39" s="15" t="n"/>
-      <c r="J39" s="15" t="n"/>
-    </row>
-    <row r="40" ht="74" customHeight="1">
-      <c r="A40" s="17" t="inlineStr">
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="15" t="n"/>
+      <c r="I42" s="15" t="n"/>
+      <c r="J42" s="15" t="n"/>
+    </row>
+    <row r="43" ht="74" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>9.1</t>
         </is>
       </c>
-      <c r="B40" s="18" t="inlineStr">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>View who is out on the team calendar</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
+      <c r="C43" s="18" t="inlineStr">
         <is>
           <t>Approver</t>
         </is>
       </c>
-      <c r="D40" s="18" t="inlineStr">
+      <c r="D43" s="18" t="inlineStr">
         <is>
           <t>Open Team Leave Calendar.
 Look at the month view, then the week view.
@@ -2391,204 +2545,207 @@
 Click View all upcoming leaves.</t>
         </is>
       </c>
-      <c r="E40" s="18" t="inlineStr">
+      <c r="E43" s="18" t="inlineStr">
         <is>
           <t>Approved leaves (and converted leaves) for the team appear on the calendar.
 Leaves that are still pending, rejected, or cancelled do not appear.
 The upcoming list shows approved leaves that start after today.</t>
         </is>
       </c>
-      <c r="F40" s="18" t="inlineStr">
+      <c r="F43" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G40" s="11" t="inlineStr"/>
-      <c r="H40" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I40" s="11" t="inlineStr"/>
-      <c r="J40" s="11" t="inlineStr"/>
-    </row>
-    <row r="41" ht="24" customHeight="1">
-      <c r="A41" s="15" t="n"/>
-      <c r="B41" s="16" t="inlineStr">
+      <c r="G43" s="11" t="inlineStr"/>
+      <c r="H43" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr"/>
+      <c r="J43" s="11" t="inlineStr"/>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="15" t="n"/>
+      <c r="B44" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  10.  Notifications and activity history</t>
         </is>
       </c>
-      <c r="C41" s="15" t="n"/>
-      <c r="D41" s="15" t="n"/>
-      <c r="E41" s="15" t="n"/>
-      <c r="F41" s="15" t="n"/>
-      <c r="G41" s="15" t="n"/>
-      <c r="H41" s="15" t="n"/>
-      <c r="I41" s="15" t="n"/>
-      <c r="J41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="60" customHeight="1">
-      <c r="A42" s="22" t="inlineStr">
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="15" t="n"/>
+      <c r="H44" s="15" t="n"/>
+      <c r="I44" s="15" t="n"/>
+      <c r="J44" s="15" t="n"/>
+    </row>
+    <row r="45" ht="88" customHeight="1">
+      <c r="A45" s="22" t="inlineStr">
         <is>
           <t>10.1</t>
         </is>
       </c>
-      <c r="B42" s="23" t="inlineStr">
-        <is>
-          <t>Notification bell</t>
-        </is>
-      </c>
-      <c r="C42" s="23" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>Header bell icon (should be removed)</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="inlineStr">
         <is>
           <t>Any user</t>
         </is>
       </c>
-      <c r="D42" s="23" t="inlineStr">
-        <is>
-          <t>Click the bell icon at the top of the page. Try Mark all as read and click an item.</t>
-        </is>
-      </c>
-      <c r="E42" s="23" t="inlineStr">
-        <is>
-          <t>A list opens, but the items are sample messages only.
-They do not update when you approve or reject a real leave.
-Do not treat this as a failed test.</t>
-        </is>
-      </c>
-      <c r="F42" s="23" t="inlineStr">
-        <is>
-          <t>Real updates are sent by email, not by this bell.</t>
-        </is>
-      </c>
-      <c r="G42" s="11" t="inlineStr"/>
-      <c r="H42" s="24" t="inlineStr">
+      <c r="D45" s="23" t="inlineStr">
+        <is>
+          <t>Look at the top of the page.
+Note whether a bell icon is still visible.
+Do not treat this as a finished notification feature. You do not need to click through the list as a working test.</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="inlineStr">
+        <is>
+          <t>The bell should not be in the final screens.
+If it is still visible, record that it is still present and needs to be removed.
+Any messages in it are sample data only and are not real updates.
+Mark this item Pending Development — not Fail.</t>
+        </is>
+      </c>
+      <c r="F45" s="23" t="inlineStr">
+        <is>
+          <t>Real updates are sent by email, not by this icon.</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="24" t="inlineStr">
         <is>
           <t>Pending Development</t>
         </is>
       </c>
-      <c r="I42" s="11" t="inlineStr"/>
-      <c r="J42" s="11" t="inlineStr"/>
-    </row>
-    <row r="43" ht="74" customHeight="1">
-      <c r="A43" s="20" t="inlineStr">
+      <c r="I45" s="11" t="inlineStr"/>
+      <c r="J45" s="11" t="inlineStr"/>
+    </row>
+    <row r="46" ht="74" customHeight="1">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>10.2</t>
         </is>
       </c>
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B46" s="21" t="inlineStr">
         <is>
           <t>My Activity Log</t>
         </is>
       </c>
-      <c r="C43" s="21" t="inlineStr">
+      <c r="C46" s="21" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="D43" s="21" t="inlineStr">
+      <c r="D46" s="21" t="inlineStr">
         <is>
           <t>Open Activity Log.
 Filter by leave type if you want.
 Look for the leaves you filed, cancelled, or converted in this test.</t>
         </is>
       </c>
-      <c r="E43" s="21" t="inlineStr">
+      <c r="E46" s="21" t="inlineStr">
         <is>
           <t>You see a timeline of your own leave actions (submitted, approved, cancelled, conversion, and so on).
 You do not see other people’s leaves or company-wide credit grants here.</t>
         </is>
       </c>
-      <c r="F43" s="21" t="inlineStr">
+      <c r="F46" s="21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G43" s="11" t="inlineStr"/>
-      <c r="H43" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I43" s="11" t="inlineStr"/>
-      <c r="J43" s="11" t="inlineStr"/>
-    </row>
-    <row r="44" ht="60" customHeight="1">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="G46" s="11" t="inlineStr"/>
+      <c r="H46" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr"/>
+      <c r="J46" s="11" t="inlineStr"/>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>10.3</t>
         </is>
       </c>
-      <c r="B44" s="18" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Administrative Log</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D44" s="18" t="inlineStr">
+      <c r="D47" s="18" t="inlineStr">
         <is>
           <t>Open Administrative Log.
 Search for the employee you used in the test.
 Filter by group, leave type, or month if needed.</t>
         </is>
       </c>
-      <c r="E44" s="18" t="inlineStr">
+      <c r="E47" s="18" t="inlineStr">
         <is>
           <t>You see leave actions across the company, including the ones from this test.
 Credit adjustments and credit distributions also appear here.</t>
         </is>
       </c>
-      <c r="F44" s="18" t="inlineStr">
+      <c r="F47" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr"/>
-      <c r="H44" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I44" s="11" t="inlineStr"/>
-      <c r="J44" s="11" t="inlineStr"/>
-    </row>
-    <row r="45" ht="24" customHeight="1">
-      <c r="A45" s="15" t="n"/>
-      <c r="B45" s="16" t="inlineStr">
+      <c r="G47" s="11" t="inlineStr"/>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr"/>
+      <c r="J47" s="11" t="inlineStr"/>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="15" t="n"/>
+      <c r="B48" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  11.  Admin — reminders, balances, and credit distribution</t>
         </is>
       </c>
-      <c r="C45" s="15" t="n"/>
-      <c r="D45" s="15" t="n"/>
-      <c r="E45" s="15" t="n"/>
-      <c r="F45" s="15" t="n"/>
-      <c r="G45" s="15" t="n"/>
-      <c r="H45" s="15" t="n"/>
-      <c r="I45" s="15" t="n"/>
-      <c r="J45" s="15" t="n"/>
-    </row>
-    <row r="46" ht="96" customHeight="1">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="15" t="n"/>
+      <c r="H48" s="15" t="n"/>
+      <c r="I48" s="15" t="n"/>
+      <c r="J48" s="15" t="n"/>
+    </row>
+    <row r="49" ht="96" customHeight="1">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>11.1</t>
         </is>
       </c>
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B49" s="18" t="inlineStr">
         <is>
           <t>Send approval reminders</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C49" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D46" s="18" t="inlineStr">
+      <c r="D49" s="18" t="inlineStr">
         <is>
           <t>Open Leave Requests → All Leave Requests.
 If a banner shows pending approver reminders, click Send Reminder to All and confirm.
@@ -2596,46 +2753,46 @@
 Send a reminder to one approver if the button is available.</t>
         </is>
       </c>
-      <c r="E46" s="18" t="inlineStr">
+      <c r="E49" s="18" t="inlineStr">
         <is>
           <t>A success message appears after sending.
 You cannot send the same all-approvers reminder twice on the same day.
 You cannot send the same single-approver reminder twice on the same day for the same leave.</t>
         </is>
       </c>
-      <c r="F46" s="18" t="inlineStr">
+      <c r="F49" s="18" t="inlineStr">
         <is>
           <t>Waiting approvers receive a reminder email.
 Admin is not emailed even if Admin is also an approver.
 Reminders are for Vacation Leave waiting on a team approver, not for Sick Leave waiting on Admin.</t>
         </is>
       </c>
-      <c r="G46" s="11" t="inlineStr"/>
-      <c r="H46" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I46" s="11" t="inlineStr"/>
-      <c r="J46" s="11" t="inlineStr"/>
-    </row>
-    <row r="47" ht="60" customHeight="1">
-      <c r="A47" s="20" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr"/>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr"/>
+      <c r="J49" s="11" t="inlineStr"/>
+    </row>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="20" t="inlineStr">
         <is>
           <t>11.2</t>
         </is>
       </c>
-      <c r="B47" s="21" t="inlineStr">
+      <c r="B50" s="21" t="inlineStr">
         <is>
           <t>Adjust an employee’s leave credits</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C50" s="21" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D50" s="21" t="inlineStr">
         <is>
           <t>Open Leave Balances.
 Search for a test employee.
@@ -2644,44 +2801,44 @@
 Confirm.</t>
         </is>
       </c>
-      <c r="E47" s="21" t="inlineStr">
+      <c r="E50" s="21" t="inlineStr">
         <is>
           <t>A success message says the employee’s credits were updated.
 The table shows the new available days.
 The change appears later in the Administrative Log.</t>
         </is>
       </c>
-      <c r="F47" s="21" t="inlineStr">
+      <c r="F50" s="21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr"/>
-      <c r="H47" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I47" s="11" t="inlineStr"/>
-      <c r="J47" s="11" t="inlineStr"/>
-    </row>
-    <row r="48" ht="88" customHeight="1">
-      <c r="A48" s="17" t="inlineStr">
+      <c r="G50" s="11" t="inlineStr"/>
+      <c r="H50" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr"/>
+      <c r="J50" s="11" t="inlineStr"/>
+    </row>
+    <row r="51" ht="88" customHeight="1">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>11.3</t>
         </is>
       </c>
-      <c r="B48" s="18" t="inlineStr">
+      <c r="B51" s="18" t="inlineStr">
         <is>
           <t>Distribute annual leave credits</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="C51" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D48" s="18" t="inlineStr">
+      <c r="D51" s="18" t="inlineStr">
         <is>
           <t>On Leave Balances, click Distribute Leave Credits.
 Choose Annual Leave Credit Distribution and click Continue.
@@ -2689,143 +2846,145 @@
 Click Continue to Review, then Confirm Distribution.</t>
         </is>
       </c>
-      <c r="E48" s="18" t="inlineStr">
+      <c r="E51" s="18" t="inlineStr">
         <is>
           <t>A success message appears.
 Those employees’ Vacation Leave and Sick Leave available days increase.
 The Administrative Log shows that annual credits were distributed.</t>
         </is>
       </c>
-      <c r="F48" s="18" t="inlineStr">
+      <c r="F51" s="18" t="inlineStr">
         <is>
           <t>None from this action. (The notification bell may show an old sample message — ignore it.)</t>
         </is>
       </c>
-      <c r="G48" s="11" t="inlineStr"/>
-      <c r="H48" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr"/>
-      <c r="J48" s="11" t="inlineStr"/>
-    </row>
-    <row r="49" ht="56" customHeight="1">
-      <c r="A49" s="20" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr"/>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr"/>
+      <c r="J51" s="11" t="inlineStr"/>
+    </row>
+    <row r="52" ht="74" customHeight="1">
+      <c r="A52" s="20" t="inlineStr">
         <is>
           <t>11.4</t>
         </is>
       </c>
-      <c r="B49" s="21" t="inlineStr">
+      <c r="B52" s="21" t="inlineStr">
         <is>
           <t>Distribute credits to newly regularized employees</t>
         </is>
       </c>
-      <c r="C49" s="21" t="inlineStr">
+      <c r="C52" s="21" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D52" s="21" t="inlineStr">
         <is>
           <t>Distribute Leave Credits → Newly Regularized Employees.
 Select eligible people, review the amounts, and Confirm Distribution.</t>
         </is>
       </c>
-      <c r="E49" s="21" t="inlineStr">
-        <is>
-          <t>Credits are added (Vacation, Sick, PTB, and Emergency as shown on the review screen). Administrative Log is updated.</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="inlineStr">
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>Credits are added for Vacation Leave, Sick Leave, and PTB as shown on the review screen.
+Emergency Leave is not included in this distribution.
+The Administrative Log is updated.</t>
+        </is>
+      </c>
+      <c r="F52" s="21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr"/>
-      <c r="H49" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I49" s="11" t="inlineStr"/>
-      <c r="J49" s="11" t="inlineStr"/>
-    </row>
-    <row r="50" ht="60" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
+      <c r="G52" s="11" t="inlineStr"/>
+      <c r="H52" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr"/>
+      <c r="J52" s="11" t="inlineStr"/>
+    </row>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>11.5</t>
         </is>
       </c>
-      <c r="B50" s="18" t="inlineStr">
+      <c r="B53" s="18" t="inlineStr">
         <is>
           <t>Distribute credits to contractual employees</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
+      <c r="C53" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D50" s="18" t="inlineStr">
+      <c r="D53" s="18" t="inlineStr">
         <is>
           <t>Distribute Leave Credits → Contractual Employees.
 Type how many Vacation and/or Sick days to add (up to 15 each).
 Review and Confirm Distribution.</t>
         </is>
       </c>
-      <c r="E50" s="18" t="inlineStr">
+      <c r="E53" s="18" t="inlineStr">
         <is>
           <t>The typed amounts are added. Administrative Log is updated.</t>
         </is>
       </c>
-      <c r="F50" s="18" t="inlineStr">
+      <c r="F53" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G50" s="11" t="inlineStr"/>
-      <c r="H50" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I50" s="11" t="inlineStr"/>
-      <c r="J50" s="11" t="inlineStr"/>
-    </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="15" t="n"/>
-      <c r="B51" s="16" t="inlineStr">
+      <c r="G53" s="11" t="inlineStr"/>
+      <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I53" s="11" t="inlineStr"/>
+      <c r="J53" s="11" t="inlineStr"/>
+    </row>
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="15" t="n"/>
+      <c r="B54" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  12.  Admin reports</t>
         </is>
       </c>
-      <c r="C51" s="15" t="n"/>
-      <c r="D51" s="15" t="n"/>
-      <c r="E51" s="15" t="n"/>
-      <c r="F51" s="15" t="n"/>
-      <c r="G51" s="15" t="n"/>
-      <c r="H51" s="15" t="n"/>
-      <c r="I51" s="15" t="n"/>
-      <c r="J51" s="15" t="n"/>
-    </row>
-    <row r="52" ht="88" customHeight="1">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="C54" s="15" t="n"/>
+      <c r="D54" s="15" t="n"/>
+      <c r="E54" s="15" t="n"/>
+      <c r="F54" s="15" t="n"/>
+      <c r="G54" s="15" t="n"/>
+      <c r="H54" s="15" t="n"/>
+      <c r="I54" s="15" t="n"/>
+      <c r="J54" s="15" t="n"/>
+    </row>
+    <row r="55" ht="88" customHeight="1">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="B52" s="18" t="inlineStr">
+      <c r="B55" s="18" t="inlineStr">
         <is>
           <t>Monthly Attendance Report</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
+      <c r="C55" s="18" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="D55" s="18" t="inlineStr">
         <is>
           <t>Open Leave Reports → Monthly Attendance Report.
 Choose a month, a cut-off (Monthly, First Half, or Second Half), a group, and employees who had approved leave.
@@ -2833,320 +2992,320 @@
 Click Export Excel and Print.</t>
         </is>
       </c>
-      <c r="E52" s="18" t="inlineStr">
+      <c r="E55" s="18" t="inlineStr">
         <is>
           <t>The grid shows approved leave days (Vacation, Sick, Others, unpaid).
 Export Excel and Print are not ready yet and show a future-update message. That is not a failed test.</t>
         </is>
       </c>
-      <c r="F52" s="18" t="inlineStr">
+      <c r="F55" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr"/>
-      <c r="H52" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I52" s="11" t="inlineStr"/>
-      <c r="J52" s="11" t="inlineStr"/>
-    </row>
-    <row r="53" ht="56" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr"/>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I55" s="11" t="inlineStr"/>
+      <c r="J55" s="11" t="inlineStr"/>
+    </row>
+    <row r="56" ht="56" customHeight="1">
+      <c r="A56" s="22" t="inlineStr">
         <is>
           <t>12.2</t>
         </is>
       </c>
-      <c r="B53" s="23" t="inlineStr">
+      <c r="B56" s="23" t="inlineStr">
         <is>
           <t>Leave Monetization Candidates report</t>
         </is>
       </c>
-      <c r="C53" s="23" t="inlineStr">
+      <c r="C56" s="23" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D53" s="23" t="inlineStr">
+      <c r="D56" s="23" t="inlineStr">
         <is>
           <t>Open Leave Reports → Leave Monetization Candidates.
 Choose a year and click Generate Report.</t>
         </is>
       </c>
-      <c r="E53" s="23" t="inlineStr">
+      <c r="E56" s="23" t="inlineStr">
         <is>
           <t>A report may appear, but it uses sample data, not live employee records.
 Do not treat this as a failed test.</t>
         </is>
       </c>
-      <c r="F53" s="23" t="inlineStr">
+      <c r="F56" s="23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr"/>
-      <c r="H53" s="24" t="inlineStr">
+      <c r="G56" s="11" t="inlineStr"/>
+      <c r="H56" s="24" t="inlineStr">
         <is>
           <t>Pending Development</t>
         </is>
       </c>
-      <c r="I53" s="11" t="inlineStr"/>
-      <c r="J53" s="11" t="inlineStr"/>
-    </row>
-    <row r="54" ht="56" customHeight="1">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="I56" s="11" t="inlineStr"/>
+      <c r="J56" s="11" t="inlineStr"/>
+    </row>
+    <row r="57" ht="56" customHeight="1">
+      <c r="A57" s="22" t="inlineStr">
         <is>
           <t>12.3</t>
         </is>
       </c>
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B57" s="23" t="inlineStr">
         <is>
           <t>Employees with LWOP report</t>
         </is>
       </c>
-      <c r="C54" s="23" t="inlineStr">
+      <c r="C57" s="23" t="inlineStr">
         <is>
           <t>Admin</t>
         </is>
       </c>
-      <c r="D54" s="23" t="inlineStr">
+      <c r="D57" s="23" t="inlineStr">
         <is>
           <t>Open Leave Reports → Employees with LWOP.
 Choose a year and click Generate Report.</t>
         </is>
       </c>
-      <c r="E54" s="23" t="inlineStr">
+      <c r="E57" s="23" t="inlineStr">
         <is>
           <t>A report may appear, but it uses sample data, not live records.
 Do not treat this as a failed test.</t>
         </is>
       </c>
-      <c r="F54" s="23" t="inlineStr">
+      <c r="F57" s="23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G54" s="11" t="inlineStr"/>
-      <c r="H54" s="24" t="inlineStr">
+      <c r="G57" s="11" t="inlineStr"/>
+      <c r="H57" s="24" t="inlineStr">
         <is>
           <t>Pending Development</t>
         </is>
       </c>
-      <c r="I54" s="11" t="inlineStr"/>
-      <c r="J54" s="11" t="inlineStr"/>
-    </row>
-    <row r="55" ht="36" customHeight="1">
-      <c r="A55" s="15" t="n"/>
-      <c r="B55" s="16" t="inlineStr">
+      <c r="I57" s="11" t="inlineStr"/>
+      <c r="J57" s="11" t="inlineStr"/>
+    </row>
+    <row r="58" ht="36" customHeight="1">
+      <c r="A58" s="15" t="n"/>
+      <c r="B58" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  13.  Who can open which pages    —    Do not use the sign-in page for this. Just switch to a user who is only an employee, then to a user who is not Admin.</t>
         </is>
       </c>
-      <c r="C55" s="15" t="n"/>
-      <c r="D55" s="15" t="n"/>
-      <c r="E55" s="15" t="n"/>
-      <c r="F55" s="15" t="n"/>
-      <c r="G55" s="15" t="n"/>
-      <c r="H55" s="15" t="n"/>
-      <c r="I55" s="15" t="n"/>
-      <c r="J55" s="15" t="n"/>
-    </row>
-    <row r="56" ht="60" customHeight="1">
-      <c r="A56" s="17" t="inlineStr">
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="15" t="n"/>
+      <c r="E58" s="15" t="n"/>
+      <c r="F58" s="15" t="n"/>
+      <c r="G58" s="15" t="n"/>
+      <c r="H58" s="15" t="n"/>
+      <c r="I58" s="15" t="n"/>
+      <c r="J58" s="15" t="n"/>
+    </row>
+    <row r="59" ht="60" customHeight="1">
+      <c r="A59" s="17" t="inlineStr">
         <is>
           <t>13.1</t>
         </is>
       </c>
-      <c r="B56" s="18" t="inlineStr">
+      <c r="B59" s="18" t="inlineStr">
         <is>
           <t>Employee cannot open Approver pages</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
+      <c r="C59" s="18" t="inlineStr">
         <is>
           <t>Employee (not an approver)</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D59" s="18" t="inlineStr">
         <is>
           <t>As an employee who is not an approver, look at the left menu.
 Confirm Team Management is hidden.
 If you can, try opening Leave Approvals from a saved link.</t>
         </is>
       </c>
-      <c r="E56" s="18" t="inlineStr">
+      <c r="E59" s="18" t="inlineStr">
         <is>
           <t>Team Management is not in the menu. Approver pages send you back to the Dashboard.</t>
         </is>
       </c>
-      <c r="F56" s="18" t="inlineStr">
+      <c r="F59" s="18" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G56" s="11" t="inlineStr"/>
-      <c r="H56" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr"/>
-      <c r="J56" s="11" t="inlineStr"/>
-    </row>
-    <row r="57" ht="60" customHeight="1">
-      <c r="A57" s="20" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr"/>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="inlineStr"/>
+      <c r="J59" s="11" t="inlineStr"/>
+    </row>
+    <row r="60" ht="60" customHeight="1">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>13.2</t>
         </is>
       </c>
-      <c r="B57" s="21" t="inlineStr">
+      <c r="B60" s="21" t="inlineStr">
         <is>
           <t>Non-admin cannot open Admin pages</t>
         </is>
       </c>
-      <c r="C57" s="21" t="inlineStr">
+      <c r="C60" s="21" t="inlineStr">
         <is>
           <t>Employee or Approver (not Admin)</t>
         </is>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>As a user who is not Admin, look at the left menu.
 Confirm Administration is hidden.
 If you can, try opening Leave Requests (Admin) from a saved link.</t>
         </is>
       </c>
-      <c r="E57" s="21" t="inlineStr">
+      <c r="E60" s="21" t="inlineStr">
         <is>
           <t>Administration is not in the menu. Admin pages send you back to the Dashboard.</t>
         </is>
       </c>
-      <c r="F57" s="21" t="inlineStr">
+      <c r="F60" s="21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr"/>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="I57" s="11" t="inlineStr"/>
-      <c r="J57" s="11" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr">
+      <c r="G60" s="11" t="inlineStr"/>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr"/>
+      <c r="J60" s="11" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  How to use Test Status</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="26" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="B60" s="27" t="inlineStr">
+      <c r="B63" s="27" t="inlineStr">
         <is>
           <t>Worked as described.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="28" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="B61" s="27" t="inlineStr">
+      <c r="B64" s="27" t="inlineStr">
         <is>
           <t>This feature should work, but it did not.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="22" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="22" t="inlineStr">
         <is>
           <t>Pending Development</t>
         </is>
       </c>
-      <c r="B62" s="27" t="inlineStr">
+      <c r="B65" s="27" t="inlineStr">
         <is>
           <t>Not finished yet or still showing sample data. Not a fail.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="29" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="29" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="B63" s="27" t="inlineStr">
+      <c r="B66" s="27" t="inlineStr">
         <is>
           <t>Could not run (missing user, credits, or email).</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="30" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="30" t="inlineStr">
         <is>
           <t>Not Applicable</t>
         </is>
       </c>
-      <c r="B64" s="27" t="inlineStr">
+      <c r="B67" s="27" t="inlineStr">
         <is>
           <t>Does not apply to this person or this run.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="31" t="inlineStr">
-        <is>
-          <t>Not Yet Tested</t>
-        </is>
-      </c>
-      <c r="B65" s="27" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>Not Yet Tested</t>
+        </is>
+      </c>
+      <c r="B68" s="27" t="inlineStr">
         <is>
           <t>Not done yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J57"/>
+  <autoFilter ref="A4:J60"/>
   <mergeCells count="26">
-    <mergeCell ref="B61:J61"/>
-    <mergeCell ref="B60:J60"/>
-    <mergeCell ref="B17:J17"/>
-    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="B67:J67"/>
+    <mergeCell ref="B42:J42"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="A62:J62"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B44:J44"/>
     <mergeCell ref="F3:G3"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="A59:J59"/>
     <mergeCell ref="B65:J65"/>
-    <mergeCell ref="B55:J55"/>
     <mergeCell ref="A3:B3"/>
+    <mergeCell ref="B68:J68"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="B64:J64"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="B5:J5"/>
-    <mergeCell ref="B20:J20"/>
-    <mergeCell ref="B51:J51"/>
-    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B32:J32"/>
     <mergeCell ref="B63:J63"/>
-    <mergeCell ref="B41:J41"/>
-    <mergeCell ref="B62:J62"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B54:J54"/>
     <mergeCell ref="B7:J7"/>
-    <mergeCell ref="B25:J25"/>
-    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B66:J66"/>
+    <mergeCell ref="B18:J18"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B58:J58"/>
     <mergeCell ref="C3:D3"/>
-    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B48:J48"/>
   </mergeCells>
-  <conditionalFormatting sqref="H6:H57">
+  <conditionalFormatting sqref="H6:H60">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3164,7 +3323,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H6:H57" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Test Status" error="Please choose a status from the list." type="list" errorStyle="warning">
+    <dataValidation sqref="H6:H60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Test Status" error="Please choose a status from the list." type="list" errorStyle="warning">
       <formula1>"Pass,Fail,Pending Development,Blocked,Not Applicable,Not Yet Tested"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3289,7 +3448,7 @@
         </is>
       </c>
       <c r="C14" s="35">
-        <f>COUNTA('Test Checklist'!A6:A57)</f>
+        <f>COUNTA('Test Checklist'!A6:A60)</f>
         <v/>
       </c>
     </row>
@@ -3300,7 +3459,7 @@
         </is>
       </c>
       <c r="C15" s="36">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Pass")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -3311,7 +3470,7 @@
         </is>
       </c>
       <c r="C16" s="37">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Fail")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -3322,7 +3481,7 @@
         </is>
       </c>
       <c r="C17" s="38">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Pending Development")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Pending Development")</f>
         <v/>
       </c>
     </row>
@@ -3333,7 +3492,7 @@
         </is>
       </c>
       <c r="C18" s="39">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Blocked")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -3344,7 +3503,7 @@
         </is>
       </c>
       <c r="C19" s="35">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Not Applicable")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Not Applicable")</f>
         <v/>
       </c>
     </row>
@@ -3355,7 +3514,7 @@
         </is>
       </c>
       <c r="C20" s="35">
-        <f>COUNTIF('Test Checklist'!H6:H57,"Not Yet Tested")</f>
+        <f>COUNTIF('Test Checklist'!H6:H60,"Not Yet Tested")</f>
         <v/>
       </c>
     </row>
@@ -3561,7 +3720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E16"/>
+  <dimension ref="B2:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3616,12 +3775,12 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Bell icon at the top of every page</t>
+          <t>Bell icon at the top of the page</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Opens a list of sample messages. It does not update when a real leave is approved or rejected. Real updates are sent by email.</t>
+          <t>This icon should be removed from the final screens. It is still visible today and only shows sample messages. Do not test it as a working notification list.</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
@@ -3655,17 +3814,17 @@
     <row r="8" ht="48" customHeight="1">
       <c r="B8" s="41" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>12.1 (part)</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>File Leave → Leave Type list</t>
+          <t>Monthly Attendance Report — Export Excel and Print</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Long Leave is not offered in the list yet, so you cannot file it from the screen.</t>
+          <t>The report grid itself works. Export and Print show a “future update” message.</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
@@ -3677,17 +3836,17 @@
     <row r="9" ht="48" customHeight="1">
       <c r="B9" s="41" t="inlineStr">
         <is>
-          <t>12.1 (part)</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Monthly Attendance Report — Export Excel and Print</t>
+          <t>Leave Reports → Leave Monetization Candidates</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>The report grid itself works. Export and Print show a “future update” message.</t>
+          <t>Generate Report uses sample data, not live employee records.</t>
         </is>
       </c>
       <c r="E9" s="24" t="inlineStr">
@@ -3699,17 +3858,17 @@
     <row r="10" ht="48" customHeight="1">
       <c r="B10" s="41" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Leave Reports → Leave Monetization Candidates</t>
+          <t>Leave Reports → Employees with LWOP</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Generate Report uses sample data, not live employee records.</t>
+          <t>Generate Report uses sample data, not live records.</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
@@ -3721,17 +3880,17 @@
     <row r="11" ht="48" customHeight="1">
       <c r="B11" s="41" t="inlineStr">
         <is>
-          <t>12.3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>Leave Reports → Employees with LWOP</t>
+          <t>Add or remove conversion files after you already submitted a conversion</t>
         </is>
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Generate Report uses sample data, not live records.</t>
+          <t>You can attach files when you first request the conversion. Changing those files later is not available on the screen yet.</t>
         </is>
       </c>
       <c r="E11" s="24" t="inlineStr">
@@ -3748,12 +3907,12 @@
       </c>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>Add or remove conversion files after you already submitted a conversion</t>
+          <t>Undo / reverse an already approved leave</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>You can attach files when you first request the conversion. Changing those files later is not available on the screen yet.</t>
+          <t>There is no Admin action yet to reverse a confirmed leave and put the days back.</t>
         </is>
       </c>
       <c r="E12" s="24" t="inlineStr">
@@ -3770,12 +3929,12 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Undo / reverse an already approved leave</t>
+          <t>File leave on behalf of a top-level (P4) employee</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>There is no Admin action yet to reverse a confirmed leave and put the days back.</t>
+          <t>This path is not available yet.</t>
         </is>
       </c>
       <c r="E13" s="24" t="inlineStr">
@@ -3784,30 +3943,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="B14" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>File leave on behalf of a top-level (P4) employee</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>This path is not available yet.</t>
-        </is>
-      </c>
-      <c r="E14" s="24" t="inlineStr">
-        <is>
-          <t>Pending Development</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="42" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="42" t="inlineStr">
         <is>
           <t>If something on this list starts working during your test, you may still mark that checklist item Pass and note it in Remarks.</t>
         </is>
@@ -3815,9 +3952,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B15:E15"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B16:E16"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>

<commit_message>
Clarify that approvers file short-notice 3+ day VL.
The checklist now treats employee-blocked Vacation Leave of 3 or more days (start date less than one month away) and File Leave for Member as one intended path.

Co-authored-by: kdtdev06 <kdtdev06@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/Leave_Forms_Initial_System_Test_Checklist.xlsx
+++ b/docs/Leave_Forms_Initial_System_Test_Checklist.xlsx
@@ -707,7 +707,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:C30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -871,8 +871,8 @@
     <row r="27" ht="130" customHeight="1">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>• When you file Vacation Leave for yourself, use 1 or 2 working days first. Three or more consecutive working days must start at least one month later, or the form will stop you.
-• An approver filing leave for a team member can file 3 or more Vacation Leave days even if the start date is less than one month away. That is expected.
+          <t>• A regular employee cannot file Vacation Leave of 3 or more days if the start date is less than one month away. The form will stop them. The approver must file that request using File Leave for Member (items 2.6 and 8.2).
+• For your own Vacation Leave in the main happy path, use 1 or 2 working days so the one-month rule does not apply.
 • Long Leave is available. It must last between 1 and 3 calendar months, needs a supporting document, and is always unpaid. There is no 5-year service rule and no waiting period after a previous Long Leave.
 • You cannot file a second Long Leave while another Long Leave is still waiting for approval.
 • Do not pick dates that overlap another open or approved leave.
@@ -947,7 +947,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J68"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -1134,7 +1134,7 @@
       <c r="A7" s="15" t="n"/>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2.  File a Vacation Leave and get it approved    —    This is the main path. Use 1 or 2 working days so the form does not block you for filing too close to the start date.</t>
+          <t xml:space="preserve">  2.  File a Vacation Leave and get it approved    —    This is the main path. When filing for yourself, use 1 or 2 working days. A regular employee cannot file 3 or more Vacation Leave days that start less than one month from today — the approver must file that request (item 2.6).</t>
         </is>
       </c>
       <c r="C7" s="15" t="n"/>
@@ -1380,7 +1380,7 @@
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
     </row>
-    <row r="13" ht="74" customHeight="1">
+    <row r="13" ht="96" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
           <t>2.6</t>
@@ -1388,32 +1388,39 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>File your own Vacation Leave of 3 or more days too soon</t>
+          <t>3 or more Vacation Leave days starting in less than one month</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>Employee</t>
+          <t>Employee, then Approver</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Go to File Leave.
+          <t>As the regular employee, go to File Leave.
 Leave Type: Vacation Leave. Day Type: Whole day.
 Pick 3 or more consecutive working days that start less than one month from today.
-Enter a Reason and click Submit Request.</t>
+Enter a Reason and try Submit Request.
+Then switch to that employee’s Approver.
+Open File Leave for Member.
+Select the same employee.
+File the same Vacation Leave (3 or more working days, start date less than one month from today).
+Submit the request.</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>The form does not allow you to submit.
-A warning explains that leave of 3 or more consecutive days must be filed at least 1 month before the start date.
-No new leave request is created.</t>
+          <t>The regular employee cannot submit. A warning says 3 or more consecutive days must be filed at least 1 month before the start date, and tells them to ask their approver to file it.
+No leave request is created from the employee’s attempt.
+The approver can submit the same dates using File Leave for Member.
+A note may appear that this short-notice filing is allowed because the approver is filing for a member.
+The leave appears on the employee’s Dashboard as Pending Approval, filed by the approver.</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
         <is>
-          <t>None — the request should not be sent.</t>
+          <t>None from the employee’s blocked attempt. After the approver submits, the person who needs to approve that member’s leave should receive the waiting-for-approval email.</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr"/>
@@ -2358,7 +2365,7 @@
       <c r="A38" s="15" t="n"/>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8.  File leave for a team member    —    The approver files on behalf of someone in their group. A higher-level approver (or the usual approver for that person) still needs to approve it.</t>
+          <t xml:space="preserve">  8.  File leave for a team member    —    The approver files on behalf of someone in their group. This is also the only way to file a regular employee’s 3 or more day Vacation Leave when the start date is less than one month away. A higher-level approver (or the usual approver for that person) still needs to approve it.</t>
         </is>
       </c>
       <c r="C38" s="15" t="n"/>
@@ -2423,7 +2430,7 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>File 3 or more Vacation Leave days for a member, less than one month in advance</t>
+          <t>Approver files the employee’s short-notice 3+ day Vacation Leave</t>
         </is>
       </c>
       <c r="C40" s="21" t="inlineStr">
@@ -2433,8 +2440,9 @@
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>Open File Leave for Member.
-Select a Group and an Employee.
+          <t>If you already completed item 2.6 with the Approver step, mark this Pass and skip.
+Otherwise: Open File Leave for Member.
+Select a Group and a regular employee (not yourself).
 Leave Type: Vacation Leave. Day Type: Whole day.
 Pick 3 or more consecutive working days that start less than one month from today.
 Enter a Reason and Submit Request.</t>
@@ -2442,8 +2450,9 @@
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>The request is submitted successfully. The one-month advance rule does not apply when an approver files for a member.
-The leave appears on the member’s Dashboard as Pending Approval.
+          <t>This is the official way to file that request. A regular employee cannot file it on File Leave.
+The approver’s form allows submit. The one-month rule does not block File Leave for Member.
+The leave appears on the member’s Dashboard as Pending Approval, filed by the approver.
 Reserved Vacation Leave credits are held for the member, if they have enough credits. Extra days may be treated as unpaid.</t>
         </is>
       </c>
@@ -3349,7 +3358,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:E45"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
@@ -3721,7 +3730,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:E15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>

</xml_diff>